<commit_message>
DEGS1-2 DD and DPE for DEGS/BGS
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_DEGS1_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_DEGS1_INES.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>index</t>
   </si>
@@ -44,13 +44,49 @@
   </si>
   <si>
     <t>decimal</t>
+  </si>
+  <si>
+    <t>LBglyc</t>
+  </si>
+  <si>
+    <t>LBchol</t>
+  </si>
+  <si>
+    <t>LBldl</t>
+  </si>
+  <si>
+    <t>LBhdl</t>
+  </si>
+  <si>
+    <t>UStail</t>
+  </si>
+  <si>
+    <t>Ushuef</t>
+  </si>
+  <si>
+    <t>Triglyzeride [mmol/l]</t>
+  </si>
+  <si>
+    <t>HDL-Cholesterin [mmol/l]</t>
+  </si>
+  <si>
+    <t>LDL-Cholesterin [mmol/l]</t>
+  </si>
+  <si>
+    <t>Cholesterin gesamt [mg/dl]</t>
+  </si>
+  <si>
+    <t>Taillenumfang [cm]</t>
+  </si>
+  <si>
+    <t>Hüftumfang [cm]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,6 +98,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -84,10 +127,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -98,8 +142,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -402,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="49.7265625" style="3" customWidth="1"/>
@@ -422,14 +468,80 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DEGS1: documents in Ines folder
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_DEGS1_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_DEGS1_INES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C52715-F4A7-4753-AA2F-884016B79AD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653936C2-42D9-4179-9881-F627AF742C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -46,10 +46,10 @@
     <t>decimal</t>
   </si>
   <si>
-    <t>Usbmi</t>
-  </si>
-  <si>
     <t>Body-Mass-Index [kg/m2]</t>
+  </si>
+  <si>
+    <t>USbmi</t>
   </si>
 </sst>
 </file>
@@ -123,9 +123,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -163,9 +163,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -198,26 +198,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -250,26 +233,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,10 +432,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>7</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>

</xml_diff>